<commit_message>
Polish partial multi-trade estimate workbook
</commit_message>
<xml_diff>
--- a/docs/reviews/multi-trade-summary-example.xlsx
+++ b/docs/reviews/multi-trade-summary-example.xlsx
@@ -52,7 +52,7 @@
     <font>
       <name val="맑은 고딕"/>
       <b val="1"/>
-      <sz val="13"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="맑은 고딕"/>
@@ -172,12 +172,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -656,10 +659,14 @@
       <c r="B3" s="2" t="n"/>
       <c r="C3" s="2" t="n"/>
     </row>
-    <row r="4" ht="25" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>조    건 : work_category: 주택 외 건축 (출처: 부문 기본값) · duration: 1~6개월 (출처: 명세 기본값) · contractor_type: 종합건설업 (출처: 명세 기본값) · project_scale: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>조    건 : 공사 종류: 주택 외 건축 (출처: 부문 기본값)
+공사 기간: 1~6개월 (출처: 명세 기본값)
+시공사 업종: 종합건설업 (출처: 명세 기본값)
+전체 공사 규모: 이 견적만 (출처: 명세 기본값)
+상태:부분 산정</t>
         </is>
       </c>
       <c r="B4" s="2" t="n"/>
@@ -670,10 +677,10 @@
       <c r="B5" s="2" t="n"/>
       <c r="C5" s="2" t="n"/>
     </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>견적금액 : 일금 이백일십만이백팔십구원정 (₩2,100,289)   ※ 부가가치세 포함</t>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>부분 산정 금액(미산정 항목 제외): 일금 이백일십만이백팔십구원정 (₩2,100,289)   ※ 부가가치세 포함</t>
         </is>
       </c>
       <c r="B6" s="2" t="n"/>
@@ -685,121 +692,125 @@
       <c r="C7" s="2" t="n"/>
     </row>
     <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>구 분</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>금 액(원)</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>비 고</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>재료비</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="5" t="inlineStr"/>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>포함된 재료비 0원 · 별도 공종 재료 미산정</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>노무비</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>1287847</v>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>직접 + 간접 노무비</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>경비</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="7" t="n">
         <v>249476</v>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>장비·보험료·기타경비 등</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>일반관리비</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="7" t="n">
         <v>122985</v>
       </c>
-      <c r="C12" s="5" t="inlineStr"/>
+      <c r="C12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>이윤</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B13" s="7" t="n">
         <v>249046</v>
       </c>
-      <c r="C13" s="5" t="inlineStr"/>
+      <c r="C13" s="6" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>공급가액</t>
         </is>
       </c>
-      <c r="B14" s="8" t="n">
+      <c r="B14" s="9" t="n">
         <v>1909354</v>
       </c>
-      <c r="C14" s="7" t="inlineStr"/>
+      <c r="C14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>부가가치세</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="7" t="n">
         <v>190935</v>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="9" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>합 계</t>
         </is>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="11" t="n">
         <v>2100289</v>
       </c>
-      <c r="C16" s="9" t="inlineStr"/>
+      <c r="C16" s="10" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n"/>
@@ -807,7 +818,7 @@
       <c r="C17" s="2" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>빠진 항목: 건설기계대여대금 지급보증 수수료(보증 수수료 산정 방법 확인 필요) 외 8건 — 원가계산서 "빠진 항목" 참조</t>
         </is>
@@ -821,7 +832,7 @@
       <c r="C19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>표준품셈 기준 금액 · 검토 전 참고용 · 품셈이</t>
         </is>
@@ -861,1318 +872,1318 @@
   </cols>
   <sheetData>
     <row r="1" ht="29" customHeight="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>공사원가계산서</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
+      <c r="B1" s="15" t="n"/>
+      <c r="C1" s="15" t="n"/>
+      <c r="D1" s="15" t="n"/>
+      <c r="E1" s="15" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>공사명: 복수 공종 견적</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>기준일: 2026-10-16 | 조건 요약: work_category: 주택 외 건축 (출처: 부문 기본값) · duration: 1~6개월 (출처: 명세 기본값) · contractor_type: 종합건설업 (출처: 명세 기본값) · project_scale: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="n"/>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>기준일: 2026-10-16 | 조건 요약: 공사 종류: 주택 외 건축 (출처: 부문 기본값) · 공사 기간: 1~6개월 (출처: 명세 기본값) · 시공사 업종: 종합건설업 (출처: 명세 기본값) · 전체 공사 규모: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n"/>
+      <c r="C3" s="15" t="n"/>
+      <c r="D3" s="15" t="n"/>
+      <c r="E3" s="15" t="n"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>비목</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>금액</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>구성비</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>비고(산출 근거)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>재료비</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>직접재료비</t>
         </is>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="17" t="n">
+      <c r="D5" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="15" t="inlineStr">
         <is>
           <t>포함분 0원 · 별도 공종 재료 미산정</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="n"/>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="n"/>
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>간접재료비(-)</t>
         </is>
       </c>
-      <c r="C6" s="18" t="inlineStr">
+      <c r="C6" s="19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D6" s="18" t="n"/>
-      <c r="E6" s="14" t="inlineStr"/>
+      <c r="D6" s="19" t="n"/>
+      <c r="E6" s="15" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="n"/>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="n"/>
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>작업설·부산물 등(△)(-)</t>
         </is>
       </c>
-      <c r="C7" s="18" t="inlineStr">
+      <c r="C7" s="19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="14" t="inlineStr"/>
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="15" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="n"/>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="n"/>
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="9" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>직접재료비 및 재료비 항목 합계</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>노무비</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>직접노무비</t>
         </is>
       </c>
-      <c r="C9" s="16" t="n">
+      <c r="C9" s="17" t="n">
         <v>1096040</v>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="18" t="n">
         <v>0.5218519927495692</v>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
         <is>
           <t>일위대가표 물량 기준 참고 금액</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="n"/>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="A10" s="15" t="n"/>
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>간접노무비</t>
         </is>
       </c>
-      <c r="C10" s="16" t="n">
+      <c r="C10" s="17" t="n">
         <v>191807</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="18" t="n">
         <v>0.09132409873117461</v>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="15" t="inlineStr">
         <is>
           <t>직접노무비 1,096,040원 × 17.5%</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="n"/>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n">
+      <c r="C11" s="9" t="n">
         <v>1287847</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="20" t="n">
         <v>0.6131760914807438</v>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>직접노무비 + 간접노무비</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>경비</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>직접경비</t>
         </is>
       </c>
-      <c r="C12" s="16" t="n">
+      <c r="C12" s="17" t="n">
         <v>21860</v>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="18" t="n">
         <v>0.01040809145788984</v>
       </c>
-      <c r="E12" s="14" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
         <is>
           <t>일위대가표 물량 기준 참고 금액</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="n"/>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="A13" s="15" t="n"/>
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>산재보험료</t>
         </is>
       </c>
-      <c r="C13" s="16" t="n">
+      <c r="C13" s="17" t="n">
         <v>45847</v>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="18" t="n">
         <v>0.02182890068938132</v>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
         <is>
           <t>노무비 계 1,287,847원 × 3.56%</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="n"/>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="A14" s="15" t="n"/>
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>고용보험료</t>
         </is>
       </c>
-      <c r="C14" s="16" t="n">
+      <c r="C14" s="17" t="n">
         <v>13007</v>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="18" t="n">
         <v>0.006192957254930155</v>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
         <is>
           <t>노무비 계 1,287,847원 × 1.01%</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="n"/>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="A15" s="15" t="n"/>
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>건강보험료</t>
         </is>
       </c>
-      <c r="C15" s="16" t="n">
+      <c r="C15" s="17" t="n">
         <v>39402</v>
       </c>
-      <c r="D15" s="17" t="n">
+      <c r="D15" s="18" t="n">
         <v>0.01876027537162743</v>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>직접노무비 1,096,040원 × 3.595%</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="n"/>
-      <c r="B16" s="14" t="inlineStr">
+      <c r="A16" s="15" t="n"/>
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>노인장기요양보험료</t>
         </is>
       </c>
-      <c r="C16" s="16" t="n">
+      <c r="C16" s="17" t="n">
         <v>5177</v>
       </c>
-      <c r="D16" s="17" t="n">
+      <c r="D16" s="18" t="n">
         <v>0.002464898878202</v>
       </c>
-      <c r="E16" s="14" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
         <is>
           <t>건강보험료 39,402원 × 13.14%</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="n"/>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="A17" s="15" t="n"/>
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>연금보험료</t>
         </is>
       </c>
-      <c r="C17" s="16" t="n">
+      <c r="C17" s="17" t="n">
         <v>52061</v>
       </c>
-      <c r="D17" s="17" t="n">
+      <c r="D17" s="18" t="n">
         <v>0.02478754114314744</v>
       </c>
-      <c r="E17" s="14" t="inlineStr">
+      <c r="E17" s="15" t="inlineStr">
         <is>
           <t>직접노무비 1,096,040원 × 4.75%</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="n"/>
-      <c r="B18" s="14" t="inlineStr">
+      <c r="A18" s="15" t="n"/>
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>환경보전비</t>
         </is>
       </c>
-      <c r="C18" s="16" t="n">
+      <c r="C18" s="17" t="n">
         <v>5589</v>
       </c>
-      <c r="D18" s="17" t="n">
+      <c r="D18" s="18" t="n">
         <v>0.002661062358561131</v>
       </c>
-      <c r="E18" s="14" t="inlineStr">
+      <c r="E18" s="15" t="inlineStr">
         <is>
           <t>직접공사비 1,117,900원 × 0.5%</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="n"/>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="A19" s="15" t="n"/>
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t>기타경비</t>
         </is>
       </c>
-      <c r="C19" s="16" t="n">
+      <c r="C19" s="17" t="n">
         <v>64392</v>
       </c>
-      <c r="D19" s="17" t="n">
+      <c r="D19" s="18" t="n">
         <v>0.03065863793030388</v>
       </c>
-      <c r="E19" s="14" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>재료비 + 노무비 1,287,847원 × 5%</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="n"/>
-      <c r="B20" s="14" t="inlineStr">
+      <c r="A20" s="15" t="n"/>
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>하도급대금 지급보증 수수료</t>
         </is>
       </c>
-      <c r="C20" s="16" t="n">
+      <c r="C20" s="17" t="n">
         <v>905</v>
       </c>
-      <c r="D20" s="17" t="n">
+      <c r="D20" s="18" t="n">
         <v>0.0004308930818568302</v>
       </c>
-      <c r="E20" s="14" t="inlineStr">
+      <c r="E20" s="15" t="inlineStr">
         <is>
           <t>직접공사비 1,117,900원 × 0.081%</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="n"/>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="A21" s="15" t="n"/>
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t>석면분담금</t>
         </is>
       </c>
-      <c r="C21" s="16" t="n">
+      <c r="C21" s="17" t="n">
         <v>77</v>
       </c>
-      <c r="D21" s="17" t="n">
+      <c r="D21" s="18" t="n">
         <v>3.666162132925516e-05</v>
       </c>
-      <c r="E21" s="14" t="inlineStr">
+      <c r="E21" s="15" t="inlineStr">
         <is>
           <t>노무비 1,287,847원 × 0.006%</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="n"/>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="A22" s="15" t="n"/>
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t>임금채권부담금</t>
         </is>
       </c>
-      <c r="C22" s="16" t="n">
+      <c r="C22" s="17" t="n">
         <v>1159</v>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D22" s="18" t="n">
         <v>0.0005518288197481395</v>
       </c>
-      <c r="E22" s="14" t="inlineStr">
+      <c r="E22" s="15" t="inlineStr">
         <is>
           <t>노무비 1,287,847원 × 0.09%</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="n"/>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="A23" s="21" t="n"/>
+      <c r="B23" s="21" t="inlineStr">
         <is>
           <t>퇴직공제부금비</t>
         </is>
       </c>
-      <c r="C23" s="21" t="n"/>
-      <c r="D23" s="21" t="n"/>
-      <c r="E23" s="20" t="inlineStr">
+      <c r="C23" s="22" t="n"/>
+      <c r="D23" s="22" t="n"/>
+      <c r="E23" s="21" t="inlineStr">
         <is>
           <t>제외 · 직접노무비</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="20" t="n"/>
-      <c r="B24" s="20" t="inlineStr">
+      <c r="A24" s="21" t="n"/>
+      <c r="B24" s="21" t="inlineStr">
         <is>
           <t>산업안전보건관리비</t>
         </is>
       </c>
-      <c r="C24" s="21" t="n"/>
-      <c r="D24" s="21" t="n"/>
-      <c r="E24" s="20" t="inlineStr">
+      <c r="C24" s="22" t="n"/>
+      <c r="D24" s="22" t="n"/>
+      <c r="E24" s="21" t="inlineStr">
         <is>
           <t>제외 · 재료비 + 직접노무비</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="20" t="n"/>
-      <c r="B25" s="20" t="inlineStr">
+      <c r="A25" s="21" t="n"/>
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t>공사이행보증</t>
         </is>
       </c>
-      <c r="C25" s="21" t="n"/>
-      <c r="D25" s="21" t="n"/>
-      <c r="E25" s="20" t="inlineStr">
+      <c r="C25" s="22" t="n"/>
+      <c r="D25" s="22" t="n"/>
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>제외 · 지방계약법 시행령 제51조제1항 적용 의무 대상(추정가격 300억 이상 등)만 해당</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="20" t="n"/>
-      <c r="B26" s="20" t="inlineStr">
+      <c r="A26" s="21" t="n"/>
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>건설기계대여대금 지급보증 수수료</t>
         </is>
       </c>
-      <c r="C26" s="21" t="n"/>
-      <c r="D26" s="21" t="n"/>
-      <c r="E26" s="20" t="inlineStr">
+      <c r="C26" s="22" t="n"/>
+      <c r="D26" s="22" t="n"/>
+      <c r="E26" s="21" t="inlineStr">
         <is>
           <t>미산정 · 원문 요율은 '지급보증액 발급금액' 기준이라 보증 수수료 산정 방법 확인 필요</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="7" t="n"/>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>소계</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n">
+      <c r="C27" s="9" t="n">
         <v>249476</v>
       </c>
-      <c r="D27" s="19" t="n">
+      <c r="D27" s="20" t="n">
         <v>0.1187817486069774</v>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t>직접경비 + 간접경비</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="7" t="inlineStr">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>순공사원가</t>
         </is>
       </c>
-      <c r="B28" s="7" t="n"/>
-      <c r="C28" s="8" t="n">
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="9" t="n">
         <v>1537323</v>
       </c>
-      <c r="D28" s="19" t="n">
+      <c r="D28" s="20" t="n">
         <v>0.7319578400877212</v>
       </c>
-      <c r="E28" s="7" t="inlineStr">
+      <c r="E28" s="8" t="inlineStr">
         <is>
           <t>재료비 + 노무비 계 + 경비 계</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="14" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>일반관리비</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>일반관리비</t>
         </is>
       </c>
-      <c r="C29" s="16" t="n">
+      <c r="C29" s="17" t="n">
         <v>122985</v>
       </c>
-      <c r="D29" s="17" t="n">
+      <c r="D29" s="18" t="n">
         <v>0.05855622726205775</v>
       </c>
-      <c r="E29" s="14" t="inlineStr">
+      <c r="E29" s="15" t="inlineStr">
         <is>
           <t>순공사원가 1,537,323원 × 8%</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="inlineStr">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t>이윤</t>
         </is>
       </c>
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t>이윤</t>
         </is>
       </c>
-      <c r="C30" s="16" t="n">
+      <c r="C30" s="17" t="n">
         <v>249046</v>
       </c>
-      <c r="D30" s="17" t="n">
+      <c r="D30" s="18" t="n">
         <v>0.1185770148774764</v>
       </c>
-      <c r="E30" s="14" t="inlineStr">
+      <c r="E30" s="15" t="inlineStr">
         <is>
           <t>노무비 + 경비 + 일반관리비 1,660,308원 × 15%</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>총원가</t>
         </is>
       </c>
-      <c r="B31" s="7" t="n"/>
-      <c r="C31" s="8" t="n">
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="9" t="n">
         <v>1909354</v>
       </c>
-      <c r="D31" s="19" t="n">
+      <c r="D31" s="20" t="n">
         <v>0.9090910822272554</v>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>순공사원가 + 일반관리비 + 이윤</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="14" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>부가가치세</t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>부가가치세</t>
         </is>
       </c>
-      <c r="C32" s="16" t="n">
+      <c r="C32" s="17" t="n">
         <v>190935</v>
       </c>
-      <c r="D32" s="17" t="n">
+      <c r="D32" s="18" t="n">
         <v>0.09090891777274461</v>
       </c>
-      <c r="E32" s="14" t="inlineStr">
+      <c r="E32" s="15" t="inlineStr">
         <is>
           <t>총원가 1,909,354원 × 10%</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="9" t="inlineStr">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>도급액</t>
         </is>
       </c>
-      <c r="B33" s="9" t="n"/>
-      <c r="C33" s="10" t="n">
+      <c r="B33" s="10" t="n"/>
+      <c r="C33" s="11" t="n">
         <v>2100289</v>
       </c>
-      <c r="D33" s="22" t="n">
+      <c r="D33" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="E33" s="10" t="inlineStr">
         <is>
           <t>총원가 + 부가가치세</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="20" t="inlineStr">
+      <c r="A34" s="21" t="inlineStr">
         <is>
           <t>경비</t>
         </is>
       </c>
-      <c r="B34" s="20" t="inlineStr">
+      <c r="B34" s="21" t="inlineStr">
         <is>
           <t>바탕만들기</t>
         </is>
       </c>
-      <c r="C34" s="21" t="n"/>
-      <c r="D34" s="21" t="n"/>
-      <c r="E34" s="20" t="inlineStr">
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="22" t="n"/>
+      <c r="E34" s="21" t="inlineStr">
         <is>
           <t>미산정 · 이번 계산 범위에서 미산정</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="20" t="n"/>
-      <c r="B35" s="20" t="inlineStr">
+      <c r="A35" s="21" t="n"/>
+      <c r="B35" s="21" t="inlineStr">
         <is>
           <t>비계사용시 높이별 품 할증</t>
         </is>
       </c>
-      <c r="C35" s="21" t="n"/>
-      <c r="D35" s="21" t="n"/>
-      <c r="E35" s="20" t="inlineStr">
+      <c r="C35" s="22" t="n"/>
+      <c r="D35" s="22" t="n"/>
+      <c r="E35" s="21" t="inlineStr">
         <is>
           <t>미산정 · 이번 계산 범위에서 미산정</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="20" t="n"/>
-      <c r="B36" s="20" t="inlineStr">
+      <c r="A36" s="21" t="n"/>
+      <c r="B36" s="21" t="inlineStr">
         <is>
           <t>재료량(페인트 등)</t>
         </is>
       </c>
-      <c r="C36" s="21" t="n"/>
-      <c r="D36" s="21" t="n"/>
-      <c r="E36" s="20" t="inlineStr">
+      <c r="C36" s="22" t="n"/>
+      <c r="D36" s="22" t="n"/>
+      <c r="E36" s="21" t="inlineStr">
         <is>
           <t>미산정 · 이번 계산 범위에서 미산정</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="20" t="n"/>
-      <c r="B37" s="20" t="inlineStr">
+      <c r="A37" s="21" t="n"/>
+      <c r="B37" s="21" t="inlineStr">
         <is>
           <t>모르타르 배합(시멘트, 모래) 재료량</t>
         </is>
       </c>
-      <c r="C37" s="21" t="n"/>
-      <c r="D37" s="21" t="n"/>
-      <c r="E37" s="20" t="inlineStr">
+      <c r="C37" s="22" t="n"/>
+      <c r="D37" s="22" t="n"/>
+      <c r="E37" s="21" t="inlineStr">
         <is>
           <t>미산정 · 이번 계산 범위에서 미산정</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="14" t="n"/>
-      <c r="B38" s="14" t="n"/>
-      <c r="C38" s="18" t="n"/>
-      <c r="D38" s="18" t="n"/>
-      <c r="E38" s="14" t="n"/>
+      <c r="A38" s="15" t="n"/>
+      <c r="B38" s="15" t="n"/>
+      <c r="C38" s="19" t="n"/>
+      <c r="D38" s="19" t="n"/>
+      <c r="E38" s="15" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="inlineStr">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>빠진 항목</t>
         </is>
       </c>
-      <c r="B39" s="14" t="n"/>
-      <c r="C39" s="18" t="n"/>
-      <c r="D39" s="18" t="n"/>
-      <c r="E39" s="14" t="n"/>
+      <c r="B39" s="15" t="n"/>
+      <c r="C39" s="19" t="n"/>
+      <c r="D39" s="19" t="n"/>
+      <c r="E39" s="15" t="n"/>
     </row>
     <row r="40" ht="27" customHeight="1">
-      <c r="A40" s="15" t="inlineStr">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B40" s="15" t="inlineStr">
+      <c r="B40" s="16" t="inlineStr">
         <is>
           <t>상태</t>
         </is>
       </c>
-      <c r="C40" s="15" t="inlineStr">
+      <c r="C40" s="16" t="inlineStr">
         <is>
           <t>이유</t>
         </is>
       </c>
-      <c r="D40" s="15" t="n"/>
-      <c r="E40" s="15" t="n"/>
+      <c r="D40" s="16" t="n"/>
+      <c r="E40" s="16" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="14" t="inlineStr">
+      <c r="A41" s="15" t="inlineStr">
         <is>
           <t>퇴직공제부금비</t>
         </is>
       </c>
-      <c r="B41" s="14" t="inlineStr">
+      <c r="B41" s="15" t="inlineStr">
         <is>
           <t>제외</t>
         </is>
       </c>
-      <c r="C41" s="18" t="inlineStr">
+      <c r="C41" s="19" t="inlineStr">
         <is>
           <t>추정금액 1억 미만</t>
         </is>
       </c>
-      <c r="D41" s="18" t="n"/>
-      <c r="E41" s="14" t="n"/>
+      <c r="D41" s="19" t="n"/>
+      <c r="E41" s="15" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="14" t="inlineStr">
+      <c r="A42" s="15" t="inlineStr">
         <is>
           <t>산업안전보건관리비</t>
         </is>
       </c>
-      <c r="B42" s="14" t="inlineStr">
+      <c r="B42" s="15" t="inlineStr">
         <is>
           <t>제외</t>
         </is>
       </c>
-      <c r="C42" s="18" t="inlineStr">
+      <c r="C42" s="19" t="inlineStr">
         <is>
           <t>총 공사금액 2천만원 미만</t>
         </is>
       </c>
-      <c r="D42" s="18" t="n"/>
-      <c r="E42" s="14" t="n"/>
+      <c r="D42" s="19" t="n"/>
+      <c r="E42" s="15" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="14" t="inlineStr">
+      <c r="A43" s="15" t="inlineStr">
         <is>
           <t>공사이행보증</t>
         </is>
       </c>
-      <c r="B43" s="14" t="inlineStr">
+      <c r="B43" s="15" t="inlineStr">
         <is>
           <t>제외</t>
         </is>
       </c>
-      <c r="C43" s="18" t="inlineStr">
+      <c r="C43" s="19" t="inlineStr">
         <is>
           <t>지방계약법 시행령 제51조 대상 아님</t>
         </is>
       </c>
-      <c r="D43" s="18" t="n"/>
-      <c r="E43" s="14" t="n"/>
+      <c r="D43" s="19" t="n"/>
+      <c r="E43" s="15" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="14" t="inlineStr">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>건설기계대여대금 지급보증 수수료</t>
         </is>
       </c>
-      <c r="B44" s="14" t="inlineStr">
+      <c r="B44" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="C44" s="18" t="inlineStr">
+      <c r="C44" s="19" t="inlineStr">
         <is>
           <t>보증 수수료 산정 방법 확인 필요</t>
         </is>
       </c>
-      <c r="D44" s="18" t="n"/>
-      <c r="E44" s="14" t="n"/>
+      <c r="D44" s="19" t="n"/>
+      <c r="E44" s="15" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="14" t="inlineStr">
+      <c r="A45" s="15" t="inlineStr">
         <is>
           <t>바탕만들기</t>
         </is>
       </c>
-      <c r="B45" s="14" t="inlineStr">
+      <c r="B45" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="C45" s="18" t="inlineStr">
+      <c r="C45" s="19" t="inlineStr">
         <is>
           <t>이번 계산 범위에서 미산정</t>
         </is>
       </c>
-      <c r="D45" s="18" t="n"/>
-      <c r="E45" s="14" t="n"/>
+      <c r="D45" s="19" t="n"/>
+      <c r="E45" s="15" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="14" t="inlineStr">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>비계사용시 높이별 품 할증</t>
         </is>
       </c>
-      <c r="B46" s="14" t="inlineStr">
+      <c r="B46" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="C46" s="18" t="inlineStr">
+      <c r="C46" s="19" t="inlineStr">
         <is>
           <t>이번 계산 범위에서 미산정</t>
         </is>
       </c>
-      <c r="D46" s="18" t="n"/>
-      <c r="E46" s="14" t="n"/>
+      <c r="D46" s="19" t="n"/>
+      <c r="E46" s="15" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="14" t="inlineStr">
+      <c r="A47" s="15" t="inlineStr">
         <is>
           <t>재료량(페인트 등)</t>
         </is>
       </c>
-      <c r="B47" s="14" t="inlineStr">
+      <c r="B47" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="C47" s="18" t="inlineStr">
+      <c r="C47" s="19" t="inlineStr">
         <is>
           <t>이번 계산 범위에서 미산정</t>
         </is>
       </c>
-      <c r="D47" s="18" t="n"/>
-      <c r="E47" s="14" t="n"/>
+      <c r="D47" s="19" t="n"/>
+      <c r="E47" s="15" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="14" t="inlineStr">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>모르타르 배합(시멘트, 모래) 재료량</t>
         </is>
       </c>
-      <c r="B48" s="14" t="inlineStr">
+      <c r="B48" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="C48" s="18" t="inlineStr">
+      <c r="C48" s="19" t="inlineStr">
         <is>
           <t>이번 계산 범위에서 미산정</t>
         </is>
       </c>
-      <c r="D48" s="18" t="n"/>
-      <c r="E48" s="14" t="n"/>
+      <c r="D48" s="19" t="n"/>
+      <c r="E48" s="15" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="14" t="inlineStr">
+      <c r="A49" s="15" t="inlineStr">
         <is>
           <t>w2_5 · 바탕만들기</t>
         </is>
       </c>
-      <c r="B49" s="14" t="inlineStr">
+      <c r="B49" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="C49" s="18" t="inlineStr">
+      <c r="C49" s="19" t="inlineStr">
         <is>
           <t>이번 계산 범위에서 미산정</t>
         </is>
       </c>
-      <c r="D49" s="18" t="n"/>
-      <c r="E49" s="14" t="n"/>
+      <c r="D49" s="19" t="n"/>
+      <c r="E49" s="15" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="14" t="inlineStr">
+      <c r="A50" s="15" t="inlineStr">
         <is>
           <t>w2_5 · 비계사용시 높이별 품 할증</t>
         </is>
       </c>
-      <c r="B50" s="14" t="inlineStr">
+      <c r="B50" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="C50" s="18" t="inlineStr">
+      <c r="C50" s="19" t="inlineStr">
         <is>
           <t>이번 계산 범위에서 미산정</t>
         </is>
       </c>
-      <c r="D50" s="18" t="n"/>
-      <c r="E50" s="14" t="n"/>
+      <c r="D50" s="19" t="n"/>
+      <c r="E50" s="15" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="14" t="inlineStr">
+      <c r="A51" s="15" t="inlineStr">
         <is>
           <t>w2_5 · 재료량(페인트 등)</t>
         </is>
       </c>
-      <c r="B51" s="14" t="inlineStr">
+      <c r="B51" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="C51" s="18" t="inlineStr">
+      <c r="C51" s="19" t="inlineStr">
         <is>
           <t>이번 계산 범위에서 미산정</t>
         </is>
       </c>
-      <c r="D51" s="18" t="n"/>
-      <c r="E51" s="14" t="n"/>
+      <c r="D51" s="19" t="n"/>
+      <c r="E51" s="15" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="14" t="inlineStr">
+      <c r="A52" s="15" t="inlineStr">
         <is>
           <t>w25_27 · 모르타르 배합(시멘트, 모래) 재료량</t>
         </is>
       </c>
-      <c r="B52" s="14" t="inlineStr">
+      <c r="B52" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="C52" s="18" t="inlineStr">
+      <c r="C52" s="19" t="inlineStr">
         <is>
           <t>이번 계산 범위에서 미산정</t>
         </is>
       </c>
-      <c r="D52" s="18" t="n"/>
-      <c r="E52" s="14" t="n"/>
+      <c r="D52" s="19" t="n"/>
+      <c r="E52" s="15" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="14" t="n"/>
-      <c r="B53" s="14" t="n"/>
-      <c r="C53" s="18" t="n"/>
-      <c r="D53" s="18" t="n"/>
-      <c r="E53" s="14" t="n"/>
+      <c r="A53" s="15" t="n"/>
+      <c r="B53" s="15" t="n"/>
+      <c r="C53" s="19" t="n"/>
+      <c r="D53" s="19" t="n"/>
+      <c r="E53" s="15" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="23" t="inlineStr">
+      <c r="A54" s="24" t="inlineStr">
         <is>
           <t>적용 요율 출처</t>
         </is>
       </c>
-      <c r="B54" s="23" t="n"/>
-      <c r="C54" s="24" t="n"/>
-      <c r="D54" s="24" t="n"/>
-      <c r="E54" s="14" t="n"/>
+      <c r="B54" s="24" t="n"/>
+      <c r="C54" s="25" t="n"/>
+      <c r="D54" s="25" t="n"/>
+      <c r="E54" s="15" t="n"/>
     </row>
     <row r="55" ht="27" customHeight="1">
-      <c r="A55" s="15" t="inlineStr">
+      <c r="A55" s="16" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B55" s="15" t="inlineStr">
+      <c r="B55" s="16" t="inlineStr">
         <is>
           <t>요율</t>
         </is>
       </c>
-      <c r="C55" s="15" t="inlineStr">
+      <c r="C55" s="16" t="inlineStr">
         <is>
           <t>적용 구간</t>
         </is>
       </c>
-      <c r="D55" s="15" t="inlineStr">
+      <c r="D55" s="16" t="inlineStr">
         <is>
           <t>출처</t>
         </is>
       </c>
-      <c r="E55" s="15" t="n"/>
+      <c r="E55" s="16" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="14" t="inlineStr">
+      <c r="A56" s="15" t="inlineStr">
         <is>
           <t>간접노무비</t>
         </is>
       </c>
-      <c r="B56" s="14" t="inlineStr">
+      <c r="B56" s="15" t="inlineStr">
         <is>
           <t>17.5%</t>
         </is>
       </c>
-      <c r="C56" s="18" t="inlineStr">
+      <c r="C56" s="19" t="inlineStr">
         <is>
           <t>10억 미만·6개월 이하</t>
         </is>
       </c>
-      <c r="D56" s="18" t="inlineStr">
+      <c r="D56" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E56" s="14" t="n"/>
+      <c r="E56" s="15" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="14" t="inlineStr">
+      <c r="A57" s="15" t="inlineStr">
         <is>
           <t>산재보험료</t>
         </is>
       </c>
-      <c r="B57" s="14" t="inlineStr">
+      <c r="B57" s="15" t="inlineStr">
         <is>
           <t>3.56%</t>
         </is>
       </c>
-      <c r="C57" s="18" t="inlineStr">
+      <c r="C57" s="19" t="inlineStr">
         <is>
           <t>노무비 계 기준</t>
         </is>
       </c>
-      <c r="D57" s="18" t="inlineStr">
+      <c r="D57" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E57" s="14" t="n"/>
+      <c r="E57" s="15" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="14" t="inlineStr">
+      <c r="A58" s="15" t="inlineStr">
         <is>
           <t>고용보험료</t>
         </is>
       </c>
-      <c r="B58" s="14" t="inlineStr">
+      <c r="B58" s="15" t="inlineStr">
         <is>
           <t>1.01%</t>
         </is>
       </c>
-      <c r="C58" s="18" t="inlineStr">
+      <c r="C58" s="19" t="inlineStr">
         <is>
           <t>7등급</t>
         </is>
       </c>
-      <c r="D58" s="18" t="inlineStr">
+      <c r="D58" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E58" s="14" t="n"/>
+      <c r="E58" s="15" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="14" t="inlineStr">
+      <c r="A59" s="15" t="inlineStr">
         <is>
           <t>건강보험료</t>
         </is>
       </c>
-      <c r="B59" s="14" t="inlineStr">
+      <c r="B59" s="15" t="inlineStr">
         <is>
           <t>3.595%</t>
         </is>
       </c>
-      <c r="C59" s="18" t="inlineStr">
+      <c r="C59" s="19" t="inlineStr">
         <is>
           <t>직접노무비 기준</t>
         </is>
       </c>
-      <c r="D59" s="18" t="inlineStr">
+      <c r="D59" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E59" s="14" t="n"/>
+      <c r="E59" s="15" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="14" t="inlineStr">
+      <c r="A60" s="15" t="inlineStr">
         <is>
           <t>노인장기요양보험료</t>
         </is>
       </c>
-      <c r="B60" s="14" t="inlineStr">
+      <c r="B60" s="15" t="inlineStr">
         <is>
           <t>13.14%</t>
         </is>
       </c>
-      <c r="C60" s="18" t="inlineStr">
+      <c r="C60" s="19" t="inlineStr">
         <is>
           <t>건강보험료 기준</t>
         </is>
       </c>
-      <c r="D60" s="18" t="inlineStr">
+      <c r="D60" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E60" s="14" t="n"/>
+      <c r="E60" s="15" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="14" t="inlineStr">
+      <c r="A61" s="15" t="inlineStr">
         <is>
           <t>연금보험료</t>
         </is>
       </c>
-      <c r="B61" s="14" t="inlineStr">
+      <c r="B61" s="15" t="inlineStr">
         <is>
           <t>4.75%</t>
         </is>
       </c>
-      <c r="C61" s="18" t="inlineStr">
+      <c r="C61" s="19" t="inlineStr">
         <is>
           <t>직접노무비 기준</t>
         </is>
       </c>
-      <c r="D61" s="18" t="inlineStr">
+      <c r="D61" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E61" s="14" t="n"/>
+      <c r="E61" s="15" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="14" t="inlineStr">
+      <c r="A62" s="15" t="inlineStr">
         <is>
           <t>환경보전비</t>
         </is>
       </c>
-      <c r="B62" s="14" t="inlineStr">
+      <c r="B62" s="15" t="inlineStr">
         <is>
           <t>0.5%</t>
         </is>
       </c>
-      <c r="C62" s="18" t="inlineStr">
+      <c r="C62" s="19" t="inlineStr">
         <is>
           <t>주택 외 건축</t>
         </is>
       </c>
-      <c r="D62" s="18" t="inlineStr">
+      <c r="D62" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E62" s="14" t="n"/>
+      <c r="E62" s="15" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="14" t="inlineStr">
+      <c r="A63" s="15" t="inlineStr">
         <is>
           <t>기타경비</t>
         </is>
       </c>
-      <c r="B63" s="14" t="inlineStr">
+      <c r="B63" s="15" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C63" s="18" t="inlineStr">
+      <c r="C63" s="19" t="inlineStr">
         <is>
           <t>10억 미만·6개월 이하</t>
         </is>
       </c>
-      <c r="D63" s="18" t="inlineStr">
+      <c r="D63" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E63" s="14" t="n"/>
+      <c r="E63" s="15" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="14" t="inlineStr">
+      <c r="A64" s="15" t="inlineStr">
         <is>
           <t>하도급대금 지급보증 수수료</t>
         </is>
       </c>
-      <c r="B64" s="14" t="inlineStr">
+      <c r="B64" s="15" t="inlineStr">
         <is>
           <t>0.081%</t>
         </is>
       </c>
-      <c r="C64" s="18" t="inlineStr">
+      <c r="C64" s="19" t="inlineStr">
         <is>
           <t>50억 미만</t>
         </is>
       </c>
-      <c r="D64" s="18" t="inlineStr">
+      <c r="D64" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E64" s="14" t="n"/>
+      <c r="E64" s="15" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="14" t="inlineStr">
+      <c r="A65" s="15" t="inlineStr">
         <is>
           <t>석면분담금</t>
         </is>
       </c>
-      <c r="B65" s="14" t="inlineStr">
+      <c r="B65" s="15" t="inlineStr">
         <is>
           <t>0.006%</t>
         </is>
       </c>
-      <c r="C65" s="18" t="inlineStr">
+      <c r="C65" s="19" t="inlineStr">
         <is>
           <t>노무비 기준</t>
         </is>
       </c>
-      <c r="D65" s="18" t="inlineStr">
+      <c r="D65" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E65" s="14" t="n"/>
+      <c r="E65" s="15" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="14" t="inlineStr">
+      <c r="A66" s="15" t="inlineStr">
         <is>
           <t>임금채권부담금</t>
         </is>
       </c>
-      <c r="B66" s="14" t="inlineStr">
+      <c r="B66" s="15" t="inlineStr">
         <is>
           <t>0.09%</t>
         </is>
       </c>
-      <c r="C66" s="18" t="inlineStr">
+      <c r="C66" s="19" t="inlineStr">
         <is>
           <t>노무비 기준</t>
         </is>
       </c>
-      <c r="D66" s="18" t="inlineStr">
+      <c r="D66" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E66" s="14" t="n"/>
+      <c r="E66" s="15" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="14" t="inlineStr">
+      <c r="A67" s="15" t="inlineStr">
         <is>
           <t>일반관리비</t>
         </is>
       </c>
-      <c r="B67" s="14" t="inlineStr">
+      <c r="B67" s="15" t="inlineStr">
         <is>
           <t>8%</t>
         </is>
       </c>
-      <c r="C67" s="18" t="inlineStr">
+      <c r="C67" s="19" t="inlineStr">
         <is>
           <t>50억 미만·종합</t>
         </is>
       </c>
-      <c r="D67" s="18" t="inlineStr">
+      <c r="D67" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E67" s="14" t="n"/>
+      <c r="E67" s="15" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="14" t="inlineStr">
+      <c r="A68" s="15" t="inlineStr">
         <is>
           <t>이윤</t>
         </is>
       </c>
-      <c r="B68" s="14" t="inlineStr">
+      <c r="B68" s="15" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C68" s="18" t="inlineStr">
+      <c r="C68" s="19" t="inlineStr">
         <is>
           <t>50억 미만</t>
         </is>
       </c>
-      <c r="D68" s="18" t="inlineStr">
+      <c r="D68" s="19" t="inlineStr">
         <is>
           <t>조달청 제비율 2026.4.13., 건축</t>
         </is>
       </c>
-      <c r="E68" s="14" t="n"/>
+      <c r="E68" s="15" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="14" t="inlineStr">
+      <c r="A69" s="15" t="inlineStr">
         <is>
           <t>부가가치세</t>
         </is>
       </c>
-      <c r="B69" s="14" t="inlineStr">
+      <c r="B69" s="15" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C69" s="18" t="inlineStr">
+      <c r="C69" s="19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D69" s="18" t="inlineStr">
+      <c r="D69" s="19" t="inlineStr">
         <is>
           <t>부가가치세법</t>
         </is>
       </c>
-      <c r="E69" s="14" t="n"/>
+      <c r="E69" s="15" t="n"/>
     </row>
     <row r="70" ht="23" customHeight="1">
-      <c r="A70" s="25" t="inlineStr">
+      <c r="A70" s="26" t="inlineStr">
         <is>
           <t>표준품셈 기준 금액 · 검토 전 참고용 · 품셈이</t>
         </is>
       </c>
-      <c r="B70" s="14" t="n"/>
-      <c r="C70" s="18" t="n"/>
-      <c r="D70" s="18" t="n"/>
-      <c r="E70" s="14" t="n"/>
+      <c r="B70" s="15" t="n"/>
+      <c r="C70" s="19" t="n"/>
+      <c r="D70" s="19" t="n"/>
+      <c r="E70" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="40">
@@ -2247,340 +2258,340 @@
   </cols>
   <sheetData>
     <row r="1" ht="29" customHeight="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>공사내역서</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
-      <c r="G1" s="14" t="n"/>
-      <c r="H1" s="14" t="n"/>
-      <c r="I1" s="14" t="n"/>
-      <c r="J1" s="14" t="n"/>
-      <c r="K1" s="14" t="n"/>
-      <c r="L1" s="14" t="n"/>
-      <c r="M1" s="14" t="n"/>
+      <c r="B1" s="15" t="n"/>
+      <c r="C1" s="15" t="n"/>
+      <c r="D1" s="15" t="n"/>
+      <c r="E1" s="15" t="n"/>
+      <c r="F1" s="15" t="n"/>
+      <c r="G1" s="15" t="n"/>
+      <c r="H1" s="15" t="n"/>
+      <c r="I1" s="15" t="n"/>
+      <c r="J1" s="15" t="n"/>
+      <c r="K1" s="15" t="n"/>
+      <c r="L1" s="15" t="n"/>
+      <c r="M1" s="15" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>공사명: 복수 공종 견적</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="14" t="n"/>
-      <c r="G2" s="14" t="n"/>
-      <c r="H2" s="14" t="n"/>
-      <c r="I2" s="14" t="n"/>
-      <c r="J2" s="14" t="n"/>
-      <c r="K2" s="14" t="n"/>
-      <c r="L2" s="14" t="n"/>
-      <c r="M2" s="14" t="n"/>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="15" t="n"/>
+      <c r="G2" s="15" t="n"/>
+      <c r="H2" s="15" t="n"/>
+      <c r="I2" s="15" t="n"/>
+      <c r="J2" s="15" t="n"/>
+      <c r="K2" s="15" t="n"/>
+      <c r="L2" s="15" t="n"/>
+      <c r="M2" s="15" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>기준일: 2026-10-16 | 조건 요약: work_category: 주택 외 건축 (출처: 부문 기본값) · duration: 1~6개월 (출처: 명세 기본값) · contractor_type: 종합건설업 (출처: 명세 기본값) · project_scale: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="n"/>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="14" t="n"/>
-      <c r="G3" s="14" t="n"/>
-      <c r="H3" s="14" t="n"/>
-      <c r="I3" s="14" t="n"/>
-      <c r="J3" s="14" t="n"/>
-      <c r="K3" s="14" t="n"/>
-      <c r="L3" s="14" t="n"/>
-      <c r="M3" s="14" t="n"/>
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>기준일: 2026-10-16 | 조건 요약: 공사 종류: 주택 외 건축 (출처: 부문 기본값) · 공사 기간: 1~6개월 (출처: 명세 기본값) · 시공사 업종: 종합건설업 (출처: 명세 기본값) · 전체 공사 규모: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n"/>
+      <c r="C3" s="15" t="n"/>
+      <c r="D3" s="15" t="n"/>
+      <c r="E3" s="15" t="n"/>
+      <c r="F3" s="15" t="n"/>
+      <c r="G3" s="15" t="n"/>
+      <c r="H3" s="15" t="n"/>
+      <c r="I3" s="15" t="n"/>
+      <c r="J3" s="15" t="n"/>
+      <c r="K3" s="15" t="n"/>
+      <c r="L3" s="15" t="n"/>
+      <c r="M3" s="15" t="n"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>품 명</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>규 격</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>단위</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>수량</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>재료비</t>
         </is>
       </c>
-      <c r="F4" s="15" t="n"/>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>노무비</t>
         </is>
       </c>
-      <c r="H4" s="15" t="n"/>
-      <c r="I4" s="15" t="inlineStr">
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="inlineStr">
         <is>
           <t>경비</t>
         </is>
       </c>
-      <c r="J4" s="15" t="n"/>
-      <c r="K4" s="15" t="inlineStr">
+      <c r="J4" s="16" t="n"/>
+      <c r="K4" s="16" t="inlineStr">
         <is>
           <t>합계</t>
         </is>
       </c>
-      <c r="L4" s="15" t="n"/>
-      <c r="M4" s="15" t="inlineStr">
+      <c r="L4" s="16" t="n"/>
+      <c r="M4" s="16" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
     </row>
     <row r="5" ht="27" customHeight="1">
-      <c r="A5" s="15" t="n"/>
-      <c r="B5" s="15" t="n"/>
-      <c r="C5" s="15" t="n"/>
-      <c r="D5" s="15" t="n"/>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="n"/>
+      <c r="B5" s="16" t="n"/>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>단가</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>금액</t>
         </is>
       </c>
-      <c r="G5" s="15" t="inlineStr">
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>단가</t>
         </is>
       </c>
-      <c r="H5" s="15" t="inlineStr">
+      <c r="H5" s="16" t="inlineStr">
         <is>
           <t>금액</t>
         </is>
       </c>
-      <c r="I5" s="15" t="inlineStr">
+      <c r="I5" s="16" t="inlineStr">
         <is>
           <t>단가</t>
         </is>
       </c>
-      <c r="J5" s="15" t="inlineStr">
+      <c r="J5" s="16" t="inlineStr">
         <is>
           <t>금액</t>
         </is>
       </c>
-      <c r="K5" s="15" t="inlineStr">
+      <c r="K5" s="16" t="inlineStr">
         <is>
           <t>단가</t>
         </is>
       </c>
-      <c r="L5" s="15" t="inlineStr">
+      <c r="L5" s="16" t="inlineStr">
         <is>
           <t>금액</t>
         </is>
       </c>
-      <c r="M5" s="15" t="n"/>
+      <c r="M5" s="16" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 도장 수성페인트 롤러칠 2회 벽면100㎡ 벽면</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>w2_5</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>㎡</t>
         </is>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="D6" s="27" t="n">
         <v>100</v>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="19" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="F6" s="18" t="inlineStr">
+      <c r="F6" s="19" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="G6" s="16" t="n">
+      <c r="G6" s="17" t="n">
         <v>7128</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="17" t="n">
         <v>712800</v>
       </c>
-      <c r="I6" s="16" t="n">
+      <c r="I6" s="17" t="n">
         <v>142</v>
       </c>
-      <c r="J6" s="16" t="n">
+      <c r="J6" s="17" t="n">
         <v>14200</v>
       </c>
-      <c r="K6" s="16" t="n">
+      <c r="K6" s="17" t="n">
         <v>7270</v>
       </c>
-      <c r="L6" s="16" t="n">
+      <c r="L6" s="17" t="n">
         <v>727000</v>
       </c>
-      <c r="M6" s="14" t="inlineStr">
+      <c r="M6" s="15" t="inlineStr">
         <is>
           <t>제 1호표 · PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>[w25_27] 실내 방수모르타르10㎜ 바닥20㎡ 바닥</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>w25_27</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>㎡</t>
         </is>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="D7" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="F7" s="18" t="inlineStr">
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="G7" s="16" t="n">
+      <c r="G7" s="17" t="n">
         <v>19162</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="17" t="n">
         <v>383240</v>
       </c>
-      <c r="I7" s="16" t="n">
+      <c r="I7" s="17" t="n">
         <v>383</v>
       </c>
-      <c r="J7" s="16" t="n">
+      <c r="J7" s="17" t="n">
         <v>7660</v>
       </c>
-      <c r="K7" s="16" t="n">
+      <c r="K7" s="17" t="n">
         <v>19545</v>
       </c>
-      <c r="L7" s="16" t="n">
+      <c r="L7" s="17" t="n">
         <v>390900</v>
       </c>
-      <c r="M7" s="14" t="inlineStr">
+      <c r="M7" s="15" t="inlineStr">
         <is>
           <t>제 2호표 · PARTIAL</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>합계(공종 물량 별도)</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr"/>
-      <c r="C8" s="7" t="inlineStr"/>
-      <c r="D8" s="27" t="n"/>
-      <c r="E8" s="27" t="inlineStr">
+      <c r="B8" s="8" t="inlineStr"/>
+      <c r="C8" s="8" t="inlineStr"/>
+      <c r="D8" s="28" t="n"/>
+      <c r="E8" s="28" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="F8" s="27" t="inlineStr">
+      <c r="F8" s="28" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="G8" s="27" t="n"/>
-      <c r="H8" s="8" t="n">
+      <c r="G8" s="28" t="n"/>
+      <c r="H8" s="9" t="n">
         <v>1096040</v>
       </c>
-      <c r="I8" s="27" t="n"/>
-      <c r="J8" s="8" t="n">
+      <c r="I8" s="28" t="n"/>
+      <c r="J8" s="9" t="n">
         <v>21860</v>
       </c>
-      <c r="K8" s="27" t="n"/>
-      <c r="L8" s="8" t="n">
+      <c r="K8" s="28" t="n"/>
+      <c r="L8" s="9" t="n">
         <v>1117900</v>
       </c>
-      <c r="M8" s="7" t="inlineStr">
+      <c r="M8" s="8" t="inlineStr">
         <is>
           <t>직접비 부분합계</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>미산정 항목 제외 부분 합계</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="18" t="n"/>
-      <c r="E9" s="18" t="n"/>
-      <c r="F9" s="18" t="n"/>
-      <c r="G9" s="18" t="n"/>
-      <c r="H9" s="18" t="n"/>
-      <c r="I9" s="18" t="n"/>
-      <c r="J9" s="18" t="n"/>
-      <c r="K9" s="18" t="n"/>
-      <c r="L9" s="18" t="n"/>
-      <c r="M9" s="14" t="n"/>
+      <c r="B9" s="15" t="n"/>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="19" t="n"/>
+      <c r="F9" s="19" t="n"/>
+      <c r="G9" s="19" t="n"/>
+      <c r="H9" s="19" t="n"/>
+      <c r="I9" s="19" t="n"/>
+      <c r="J9" s="19" t="n"/>
+      <c r="K9" s="19" t="n"/>
+      <c r="L9" s="19" t="n"/>
+      <c r="M9" s="15" t="n"/>
     </row>
     <row r="10" ht="23" customHeight="1">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="26" t="inlineStr">
         <is>
           <t>표준품셈 기준 금액 · 검토 전 참고용 · 품셈이</t>
         </is>
       </c>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="14" t="n"/>
-      <c r="D10" s="18" t="n"/>
-      <c r="E10" s="18" t="n"/>
-      <c r="F10" s="18" t="n"/>
-      <c r="G10" s="18" t="n"/>
-      <c r="H10" s="18" t="n"/>
-      <c r="I10" s="18" t="n"/>
-      <c r="J10" s="18" t="n"/>
-      <c r="K10" s="18" t="n"/>
-      <c r="L10" s="18" t="n"/>
-      <c r="M10" s="14" t="n"/>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="15" t="n"/>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="19" t="n"/>
+      <c r="H10" s="19" t="n"/>
+      <c r="I10" s="19" t="n"/>
+      <c r="J10" s="19" t="n"/>
+      <c r="K10" s="19" t="n"/>
+      <c r="L10" s="19" t="n"/>
+      <c r="M10" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -2629,465 +2640,465 @@
   </cols>
   <sheetData>
     <row r="1" ht="29" customHeight="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>일위대가표</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
-      <c r="G1" s="14" t="n"/>
-      <c r="H1" s="14" t="n"/>
-      <c r="I1" s="14" t="n"/>
-      <c r="J1" s="14" t="n"/>
-      <c r="K1" s="14" t="n"/>
-      <c r="L1" s="14" t="n"/>
-      <c r="M1" s="14" t="n"/>
+      <c r="B1" s="15" t="n"/>
+      <c r="C1" s="15" t="n"/>
+      <c r="D1" s="15" t="n"/>
+      <c r="E1" s="15" t="n"/>
+      <c r="F1" s="15" t="n"/>
+      <c r="G1" s="15" t="n"/>
+      <c r="H1" s="15" t="n"/>
+      <c r="I1" s="15" t="n"/>
+      <c r="J1" s="15" t="n"/>
+      <c r="K1" s="15" t="n"/>
+      <c r="L1" s="15" t="n"/>
+      <c r="M1" s="15" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>공사명: 복수 공종 견적</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="14" t="n"/>
-      <c r="G2" s="14" t="n"/>
-      <c r="H2" s="14" t="n"/>
-      <c r="I2" s="14" t="n"/>
-      <c r="J2" s="14" t="n"/>
-      <c r="K2" s="14" t="n"/>
-      <c r="L2" s="14" t="n"/>
-      <c r="M2" s="14" t="n"/>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="15" t="n"/>
+      <c r="G2" s="15" t="n"/>
+      <c r="H2" s="15" t="n"/>
+      <c r="I2" s="15" t="n"/>
+      <c r="J2" s="15" t="n"/>
+      <c r="K2" s="15" t="n"/>
+      <c r="L2" s="15" t="n"/>
+      <c r="M2" s="15" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>기준일: 2026-10-16 | 조건 요약: work_category: 주택 외 건축 (출처: 부문 기본값) · duration: 1~6개월 (출처: 명세 기본값) · contractor_type: 종합건설업 (출처: 명세 기본값) · project_scale: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="n"/>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="14" t="n"/>
-      <c r="G3" s="14" t="n"/>
-      <c r="H3" s="14" t="n"/>
-      <c r="I3" s="14" t="n"/>
-      <c r="J3" s="14" t="n"/>
-      <c r="K3" s="14" t="n"/>
-      <c r="L3" s="14" t="n"/>
-      <c r="M3" s="14" t="n"/>
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>기준일: 2026-10-16 | 조건 요약: 공사 종류: 주택 외 건축 (출처: 부문 기본값) · 공사 기간: 1~6개월 (출처: 명세 기본값) · 시공사 업종: 종합건설업 (출처: 명세 기본값) · 전체 공사 규모: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n"/>
+      <c r="C3" s="15" t="n"/>
+      <c r="D3" s="15" t="n"/>
+      <c r="E3" s="15" t="n"/>
+      <c r="F3" s="15" t="n"/>
+      <c r="G3" s="15" t="n"/>
+      <c r="H3" s="15" t="n"/>
+      <c r="I3" s="15" t="n"/>
+      <c r="J3" s="15" t="n"/>
+      <c r="K3" s="15" t="n"/>
+      <c r="L3" s="15" t="n"/>
+      <c r="M3" s="15" t="n"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>공 종</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>규 격</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>수 량</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>단 위</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>계</t>
         </is>
       </c>
-      <c r="F4" s="15" t="n"/>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>노무비</t>
         </is>
       </c>
-      <c r="H4" s="15" t="n"/>
-      <c r="I4" s="15" t="inlineStr">
+      <c r="H4" s="16" t="n"/>
+      <c r="I4" s="16" t="inlineStr">
         <is>
           <t>재료비</t>
         </is>
       </c>
-      <c r="J4" s="15" t="n"/>
-      <c r="K4" s="15" t="inlineStr">
+      <c r="J4" s="16" t="n"/>
+      <c r="K4" s="16" t="inlineStr">
         <is>
           <t>경 비</t>
         </is>
       </c>
-      <c r="L4" s="15" t="n"/>
-      <c r="M4" s="15" t="inlineStr">
+      <c r="L4" s="16" t="n"/>
+      <c r="M4" s="16" t="inlineStr">
         <is>
           <t>비 고</t>
         </is>
       </c>
     </row>
     <row r="5" ht="27" customHeight="1">
-      <c r="A5" s="15" t="n"/>
-      <c r="B5" s="15" t="n"/>
-      <c r="C5" s="15" t="n"/>
-      <c r="D5" s="15" t="n"/>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="n"/>
+      <c r="B5" s="16" t="n"/>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="16" t="n"/>
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>단가</t>
         </is>
       </c>
-      <c r="F5" s="15" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>금액</t>
         </is>
       </c>
-      <c r="G5" s="15" t="inlineStr">
+      <c r="G5" s="16" t="inlineStr">
         <is>
           <t>단가</t>
         </is>
       </c>
-      <c r="H5" s="15" t="inlineStr">
+      <c r="H5" s="16" t="inlineStr">
         <is>
           <t>금액</t>
         </is>
       </c>
-      <c r="I5" s="15" t="inlineStr">
+      <c r="I5" s="16" t="inlineStr">
         <is>
           <t>단가</t>
         </is>
       </c>
-      <c r="J5" s="15" t="inlineStr">
+      <c r="J5" s="16" t="inlineStr">
         <is>
           <t>금액</t>
         </is>
       </c>
-      <c r="K5" s="15" t="inlineStr">
+      <c r="K5" s="16" t="inlineStr">
         <is>
           <t>단가</t>
         </is>
       </c>
-      <c r="L5" s="15" t="inlineStr">
+      <c r="L5" s="16" t="inlineStr">
         <is>
           <t>금액</t>
         </is>
       </c>
-      <c r="M5" s="15" t="n"/>
+      <c r="M5" s="16" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>제 1호표 [w2_5] 도장 수성페인트 롤러칠 2회 벽면100㎡ 벽면 (㎡ 당)</t>
         </is>
       </c>
-      <c r="B6" s="7" t="n"/>
-      <c r="C6" s="27" t="n"/>
-      <c r="D6" s="7" t="n"/>
-      <c r="E6" s="27" t="n"/>
-      <c r="F6" s="8" t="n">
+      <c r="B6" s="8" t="n"/>
+      <c r="C6" s="28" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="28" t="n"/>
+      <c r="F6" s="9" t="n">
         <v>7270</v>
       </c>
-      <c r="G6" s="27" t="n"/>
-      <c r="H6" s="8" t="n">
+      <c r="G6" s="28" t="n"/>
+      <c r="H6" s="9" t="n">
         <v>7128</v>
       </c>
-      <c r="I6" s="27" t="n"/>
-      <c r="J6" s="27" t="n"/>
-      <c r="K6" s="27" t="n"/>
-      <c r="L6" s="8" t="n">
+      <c r="I6" s="28" t="n"/>
+      <c r="J6" s="28" t="n"/>
+      <c r="K6" s="28" t="n"/>
+      <c r="L6" s="9" t="n">
         <v>142</v>
       </c>
-      <c r="M6" s="7" t="n"/>
+      <c r="M6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>도장공</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr"/>
-      <c r="C7" s="26" t="n">
+      <c r="B7" s="15" t="inlineStr"/>
+      <c r="C7" s="27" t="n">
         <v>0.024</v>
       </c>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>인</t>
         </is>
       </c>
-      <c r="E7" s="18" t="n"/>
-      <c r="F7" s="16" t="n">
+      <c r="E7" s="19" t="n"/>
+      <c r="F7" s="17" t="n">
         <v>6437.4</v>
       </c>
-      <c r="G7" s="26" t="n">
+      <c r="G7" s="27" t="n">
         <v>268225</v>
       </c>
-      <c r="H7" s="16" t="n">
+      <c r="H7" s="17" t="n">
         <v>6437.4</v>
       </c>
-      <c r="I7" s="18" t="n"/>
-      <c r="J7" s="18" t="n"/>
-      <c r="K7" s="18" t="n"/>
-      <c r="L7" s="18" t="n"/>
-      <c r="M7" s="14" t="inlineStr">
+      <c r="I7" s="19" t="n"/>
+      <c r="J7" s="19" t="n"/>
+      <c r="K7" s="19" t="n"/>
+      <c r="L7" s="19" t="n"/>
+      <c r="M7" s="15" t="inlineStr">
         <is>
           <t>11-2-2 p693; 1029 p10</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>보통인부</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr"/>
-      <c r="C8" s="26" t="n">
+      <c r="B8" s="15" t="inlineStr"/>
+      <c r="C8" s="27" t="n">
         <v>0.004</v>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>인</t>
         </is>
       </c>
-      <c r="E8" s="18" t="n"/>
-      <c r="F8" s="16" t="n">
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="17" t="n">
         <v>690.7</v>
       </c>
-      <c r="G8" s="26" t="n">
+      <c r="G8" s="27" t="n">
         <v>172698</v>
       </c>
-      <c r="H8" s="16" t="n">
+      <c r="H8" s="17" t="n">
         <v>690.7</v>
       </c>
-      <c r="I8" s="18" t="n"/>
-      <c r="J8" s="18" t="n"/>
-      <c r="K8" s="18" t="n"/>
-      <c r="L8" s="18" t="n"/>
-      <c r="M8" s="14" t="inlineStr">
+      <c r="I8" s="19" t="n"/>
+      <c r="J8" s="19" t="n"/>
+      <c r="K8" s="19" t="n"/>
+      <c r="L8" s="19" t="n"/>
+      <c r="M8" s="15" t="inlineStr">
         <is>
           <t>11-2-2 p693; 1002 p10</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>공구손료 및 잡재료비</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>노무비의 2.00%</t>
         </is>
       </c>
-      <c r="C9" s="26" t="n">
+      <c r="C9" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>식</t>
         </is>
       </c>
-      <c r="E9" s="18" t="n"/>
-      <c r="F9" s="16" t="n">
+      <c r="E9" s="19" t="n"/>
+      <c r="F9" s="17" t="n">
         <v>142.5</v>
       </c>
-      <c r="G9" s="18" t="n"/>
-      <c r="H9" s="18" t="n"/>
-      <c r="I9" s="18" t="n"/>
-      <c r="J9" s="18" t="n"/>
-      <c r="K9" s="26" t="n">
+      <c r="G9" s="19" t="n"/>
+      <c r="H9" s="19" t="n"/>
+      <c r="I9" s="19" t="n"/>
+      <c r="J9" s="19" t="n"/>
+      <c r="K9" s="27" t="n">
         <v>142.5</v>
       </c>
-      <c r="L9" s="16" t="n">
+      <c r="L9" s="17" t="n">
         <v>142.5</v>
       </c>
-      <c r="M9" s="14" t="inlineStr">
+      <c r="M9" s="15" t="inlineStr">
         <is>
           <t>11-2-2 p693</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>제 2호표 [w25_27] 실내 방수모르타르10㎜ 바닥20㎡ 바닥 (㎡ 당)</t>
         </is>
       </c>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="18" t="n"/>
-      <c r="D10" s="14" t="n"/>
-      <c r="E10" s="18" t="n"/>
-      <c r="F10" s="16" t="n">
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="15" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="17" t="n">
         <v>19545</v>
       </c>
-      <c r="G10" s="18" t="n"/>
-      <c r="H10" s="16" t="n">
+      <c r="G10" s="19" t="n"/>
+      <c r="H10" s="17" t="n">
         <v>19162</v>
       </c>
-      <c r="I10" s="18" t="n"/>
-      <c r="J10" s="18" t="n"/>
-      <c r="K10" s="18" t="n"/>
-      <c r="L10" s="16" t="n">
+      <c r="I10" s="19" t="n"/>
+      <c r="J10" s="19" t="n"/>
+      <c r="K10" s="19" t="n"/>
+      <c r="L10" s="17" t="n">
         <v>383</v>
       </c>
-      <c r="M10" s="14" t="n"/>
+      <c r="M10" s="15" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>미장공</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr"/>
-      <c r="C11" s="26" t="n">
+      <c r="B11" s="15" t="inlineStr"/>
+      <c r="C11" s="27" t="n">
         <v>0.047</v>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>인</t>
         </is>
       </c>
-      <c r="E11" s="18" t="n"/>
-      <c r="F11" s="16" t="n">
+      <c r="E11" s="19" t="n"/>
+      <c r="F11" s="17" t="n">
         <v>13117.7</v>
       </c>
-      <c r="G11" s="26" t="n">
+      <c r="G11" s="27" t="n">
         <v>279102</v>
       </c>
-      <c r="H11" s="16" t="n">
+      <c r="H11" s="17" t="n">
         <v>13117.7</v>
       </c>
-      <c r="I11" s="18" t="n"/>
-      <c r="J11" s="18" t="n"/>
-      <c r="K11" s="18" t="n"/>
-      <c r="L11" s="18" t="n"/>
-      <c r="M11" s="14" t="inlineStr">
+      <c r="I11" s="19" t="n"/>
+      <c r="J11" s="19" t="n"/>
+      <c r="K11" s="19" t="n"/>
+      <c r="L11" s="19" t="n"/>
+      <c r="M11" s="15" t="inlineStr">
         <is>
           <t>6-4-3 p662; 1027 p10</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>보통인부</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr"/>
-      <c r="C12" s="26" t="n">
+      <c r="B12" s="15" t="inlineStr"/>
+      <c r="C12" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>인</t>
         </is>
       </c>
-      <c r="E12" s="18" t="n"/>
-      <c r="F12" s="16" t="n">
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="17" t="n">
         <v>6044.4</v>
       </c>
-      <c r="G12" s="26" t="n">
+      <c r="G12" s="27" t="n">
         <v>172698</v>
       </c>
-      <c r="H12" s="16" t="n">
+      <c r="H12" s="17" t="n">
         <v>6044.4</v>
       </c>
-      <c r="I12" s="18" t="n"/>
-      <c r="J12" s="18" t="n"/>
-      <c r="K12" s="18" t="n"/>
-      <c r="L12" s="18" t="n"/>
-      <c r="M12" s="14" t="inlineStr">
+      <c r="I12" s="19" t="n"/>
+      <c r="J12" s="19" t="n"/>
+      <c r="K12" s="19" t="n"/>
+      <c r="L12" s="19" t="n"/>
+      <c r="M12" s="15" t="inlineStr">
         <is>
           <t>6-4-3 p662; 1002 p10</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>공구손료 및 경장비(비빔기 등) 기계경비</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="15" t="inlineStr">
         <is>
           <t>노무비의 2.00%</t>
         </is>
       </c>
-      <c r="C13" s="26" t="n">
+      <c r="C13" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>식</t>
         </is>
       </c>
-      <c r="E13" s="18" t="n"/>
-      <c r="F13" s="16" t="n">
+      <c r="E13" s="19" t="n"/>
+      <c r="F13" s="17" t="n">
         <v>383.2</v>
       </c>
-      <c r="G13" s="18" t="n"/>
-      <c r="H13" s="18" t="n"/>
-      <c r="I13" s="18" t="n"/>
-      <c r="J13" s="18" t="n"/>
-      <c r="K13" s="26" t="n">
+      <c r="G13" s="19" t="n"/>
+      <c r="H13" s="19" t="n"/>
+      <c r="I13" s="19" t="n"/>
+      <c r="J13" s="19" t="n"/>
+      <c r="K13" s="27" t="n">
         <v>383.2</v>
       </c>
-      <c r="L13" s="16" t="n">
+      <c r="L13" s="17" t="n">
         <v>383.2</v>
       </c>
-      <c r="M13" s="14" t="inlineStr">
+      <c r="M13" s="15" t="inlineStr">
         <is>
           <t>6-4-3 p662</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>금액 0.1원 미만 버림(품셈 1-2-2)</t>
         </is>
       </c>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="14" t="n"/>
-      <c r="E14" s="18" t="n"/>
-      <c r="F14" s="18" t="n"/>
-      <c r="G14" s="18" t="n"/>
-      <c r="H14" s="18" t="n"/>
-      <c r="I14" s="18" t="n"/>
-      <c r="J14" s="18" t="n"/>
-      <c r="K14" s="18" t="n"/>
-      <c r="L14" s="18" t="n"/>
-      <c r="M14" s="14" t="n"/>
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="19" t="n"/>
+      <c r="H14" s="19" t="n"/>
+      <c r="I14" s="19" t="n"/>
+      <c r="J14" s="19" t="n"/>
+      <c r="K14" s="19" t="n"/>
+      <c r="L14" s="19" t="n"/>
+      <c r="M14" s="15" t="n"/>
     </row>
     <row r="15" ht="23" customHeight="1">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>표준품셈 기준 금액 · 검토 전 참고용 · 품셈이</t>
         </is>
       </c>
-      <c r="B15" s="14" t="n"/>
-      <c r="C15" s="18" t="n"/>
-      <c r="D15" s="14" t="n"/>
-      <c r="E15" s="18" t="n"/>
-      <c r="F15" s="18" t="n"/>
-      <c r="G15" s="18" t="n"/>
-      <c r="H15" s="18" t="n"/>
-      <c r="I15" s="18" t="n"/>
-      <c r="J15" s="18" t="n"/>
-      <c r="K15" s="18" t="n"/>
-      <c r="L15" s="18" t="n"/>
-      <c r="M15" s="14" t="n"/>
+      <c r="B15" s="15" t="n"/>
+      <c r="C15" s="19" t="n"/>
+      <c r="D15" s="15" t="n"/>
+      <c r="E15" s="19" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
+      <c r="H15" s="19" t="n"/>
+      <c r="I15" s="19" t="n"/>
+      <c r="J15" s="19" t="n"/>
+      <c r="K15" s="19" t="n"/>
+      <c r="L15" s="19" t="n"/>
+      <c r="M15" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
@@ -3132,174 +3143,174 @@
   </cols>
   <sheetData>
     <row r="1" ht="29" customHeight="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>공종별 산출 내역</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
-      <c r="G1" s="14" t="n"/>
-      <c r="H1" s="14" t="n"/>
-      <c r="I1" s="14" t="n"/>
+      <c r="B1" s="15" t="n"/>
+      <c r="C1" s="15" t="n"/>
+      <c r="D1" s="15" t="n"/>
+      <c r="E1" s="15" t="n"/>
+      <c r="F1" s="15" t="n"/>
+      <c r="G1" s="15" t="n"/>
+      <c r="H1" s="15" t="n"/>
+      <c r="I1" s="15" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>공사명: 복수 공종 견적</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="14" t="n"/>
-      <c r="G2" s="14" t="n"/>
-      <c r="H2" s="14" t="n"/>
-      <c r="I2" s="14" t="n"/>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="15" t="n"/>
+      <c r="G2" s="15" t="n"/>
+      <c r="H2" s="15" t="n"/>
+      <c r="I2" s="15" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>기준일: 2026-10-16 | 조건 요약: work_category: 주택 외 건축 (출처: 부문 기본값) · duration: 1~6개월 (출처: 명세 기본값) · contractor_type: 종합건설업 (출처: 명세 기본값) · project_scale: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="n"/>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="14" t="n"/>
-      <c r="G3" s="14" t="n"/>
-      <c r="H3" s="14" t="n"/>
-      <c r="I3" s="14" t="n"/>
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>기준일: 2026-10-16 | 조건 요약: 공사 종류: 주택 외 건축 (출처: 부문 기본값) · 공사 기간: 1~6개월 (출처: 명세 기본값) · 시공사 업종: 종합건설업 (출처: 명세 기본값) · 전체 공사 규모: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n"/>
+      <c r="C3" s="15" t="n"/>
+      <c r="D3" s="15" t="n"/>
+      <c r="E3" s="15" t="n"/>
+      <c r="F3" s="15" t="n"/>
+      <c r="G3" s="15" t="n"/>
+      <c r="H3" s="15" t="n"/>
+      <c r="I3" s="15" t="n"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>항목 ID</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>공종</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>상태</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>수량</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>재료비</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>노무비</t>
         </is>
       </c>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>경비</t>
         </is>
       </c>
-      <c r="H4" s="15" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>직접비</t>
         </is>
       </c>
-      <c r="I4" s="15" t="inlineStr">
+      <c r="I4" s="16" t="inlineStr">
         <is>
           <t>미산정 범위</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>w2_5</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>도장 수성페인트 롤러칠 2회 벽면100㎡ 벽면</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>100㎡</t>
         </is>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="F5" s="16" t="n">
+      <c r="F5" s="17" t="n">
         <v>712800</v>
       </c>
-      <c r="G5" s="16" t="n">
+      <c r="G5" s="17" t="n">
         <v>14200</v>
       </c>
-      <c r="H5" s="16" t="n">
+      <c r="H5" s="17" t="n">
         <v>727000</v>
       </c>
-      <c r="I5" s="14" t="inlineStr">
+      <c r="I5" s="15" t="inlineStr">
         <is>
           <t>바탕만들기: 이번 계산 범위에서 미산정; 비계사용시 높이별 품 할증: 이번 계산 범위에서 미산정; 재료량(페인트 등): 이번 계산 범위에서 미산정; 바탕만들기: PDF 637쪽 11-2-2 [주] ③; 비계사용시 높이별 품 할증: PDF 637쪽 11-2-2 [주] ④; 재료량(페인트 등): PDF 637쪽 11-2-2 [주] ⑥</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>w25_27</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>실내 방수모르타르10㎜ 바닥20㎡ 바닥</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>PARTIAL</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>20㎡</t>
         </is>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="19" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
-      <c r="F6" s="16" t="n">
+      <c r="F6" s="17" t="n">
         <v>383240</v>
       </c>
-      <c r="G6" s="16" t="n">
+      <c r="G6" s="17" t="n">
         <v>7660</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="17" t="n">
         <v>390900</v>
       </c>
-      <c r="I6" s="14" t="inlineStr">
+      <c r="I6" s="15" t="inlineStr">
         <is>
           <t>모르타르 배합(시멘트, 모래) 재료량: 이번 계산 범위에서 미산정; 모르타르 배합(시멘트, 모래) 재료량: PDF 606쪽 6-4-3 [주] ②</t>
         </is>
@@ -3336,246 +3347,246 @@
   </cols>
   <sheetData>
     <row r="1" ht="29" customHeight="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>단가대비표</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
-      <c r="G1" s="14" t="n"/>
-      <c r="H1" s="14" t="n"/>
+      <c r="B1" s="15" t="n"/>
+      <c r="C1" s="15" t="n"/>
+      <c r="D1" s="15" t="n"/>
+      <c r="E1" s="15" t="n"/>
+      <c r="F1" s="15" t="n"/>
+      <c r="G1" s="15" t="n"/>
+      <c r="H1" s="15" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>공사명: 복수 공종 견적</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="14" t="n"/>
-      <c r="G2" s="14" t="n"/>
-      <c r="H2" s="14" t="n"/>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="15" t="n"/>
+      <c r="G2" s="15" t="n"/>
+      <c r="H2" s="15" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>기준일: 2026-10-16 | 조건 요약: work_category: 주택 외 건축 (출처: 부문 기본값) · duration: 1~6개월 (출처: 명세 기본값) · contractor_type: 종합건설업 (출처: 명세 기본값) · project_scale: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="n"/>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="14" t="n"/>
-      <c r="G3" s="14" t="n"/>
-      <c r="H3" s="14" t="n"/>
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>기준일: 2026-10-16 | 조건 요약: 공사 종류: 주택 외 건축 (출처: 부문 기본값) · 공사 기간: 1~6개월 (출처: 명세 기본값) · 시공사 업종: 종합건설업 (출처: 명세 기본값) · 전체 공사 규모: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n"/>
+      <c r="C3" s="15" t="n"/>
+      <c r="D3" s="15" t="n"/>
+      <c r="E3" s="15" t="n"/>
+      <c r="F3" s="15" t="n"/>
+      <c r="G3" s="15" t="n"/>
+      <c r="H3" s="15" t="n"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>품명</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>규격</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>단위</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>적용 단가</t>
         </is>
       </c>
-      <c r="F4" s="15" t="inlineStr">
+      <c r="F4" s="16" t="inlineStr">
         <is>
           <t>단가 근거</t>
         </is>
       </c>
-      <c r="G4" s="15" t="inlineStr">
+      <c r="G4" s="16" t="inlineStr">
         <is>
           <t>적용 기간</t>
         </is>
       </c>
-      <c r="H4" s="15" t="inlineStr">
+      <c r="H4" s="16" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>노임</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 도장공</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr"/>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr"/>
+      <c r="D5" s="15" t="inlineStr">
         <is>
           <t>원/인</t>
         </is>
       </c>
-      <c r="E5" s="16" t="n">
+      <c r="E5" s="17" t="n">
         <v>268225</v>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>2026년 하반기 적용 건설업 임금실태조사(대한건설협회)</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>2026 하반기</t>
         </is>
       </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>일 8시간 · 노임 코드 1029</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>노임</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 보통인부</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr"/>
-      <c r="D6" s="14" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr"/>
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>원/인</t>
         </is>
       </c>
-      <c r="E6" s="16" t="n">
+      <c r="E6" s="17" t="n">
         <v>172698</v>
       </c>
-      <c r="F6" s="14" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>2026년 하반기 적용 건설업 임금실태조사(대한건설협회)</t>
         </is>
       </c>
-      <c r="G6" s="14" t="inlineStr">
+      <c r="G6" s="15" t="inlineStr">
         <is>
           <t>2026 하반기</t>
         </is>
       </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="H6" s="15" t="inlineStr">
         <is>
           <t>일 8시간 · 노임 코드 1002</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>노임</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>[w25_27] 미장공</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr"/>
-      <c r="D7" s="14" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr"/>
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>원/인</t>
         </is>
       </c>
-      <c r="E7" s="16" t="n">
+      <c r="E7" s="17" t="n">
         <v>279102</v>
       </c>
-      <c r="F7" s="14" t="inlineStr">
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>2026년 하반기 적용 건설업 임금실태조사(대한건설협회)</t>
         </is>
       </c>
-      <c r="G7" s="14" t="inlineStr">
+      <c r="G7" s="15" t="inlineStr">
         <is>
           <t>2026 하반기</t>
         </is>
       </c>
-      <c r="H7" s="14" t="inlineStr">
+      <c r="H7" s="15" t="inlineStr">
         <is>
           <t>일 8시간 · 노임 코드 1027</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>노임</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>[w25_27] 보통인부</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr"/>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr"/>
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>원/인</t>
         </is>
       </c>
-      <c r="E8" s="16" t="n">
+      <c r="E8" s="17" t="n">
         <v>172698</v>
       </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="F8" s="15" t="inlineStr">
         <is>
           <t>2026년 하반기 적용 건설업 임금실태조사(대한건설협회)</t>
         </is>
       </c>
-      <c r="G8" s="14" t="inlineStr">
+      <c r="G8" s="15" t="inlineStr">
         <is>
           <t>2026 하반기</t>
         </is>
       </c>
-      <c r="H8" s="14" t="inlineStr">
+      <c r="H8" s="15" t="inlineStr">
         <is>
           <t>일 8시간 · 노임 코드 1002</t>
         </is>
       </c>
     </row>
     <row r="9" ht="23" customHeight="1">
-      <c r="A9" s="25" t="inlineStr">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t>표준품셈 기준 금액 · 검토 전 참고용 · 품셈이</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-      <c r="E9" s="18" t="n"/>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="n"/>
+      <c r="B9" s="15" t="n"/>
+      <c r="C9" s="15" t="n"/>
+      <c r="D9" s="15" t="n"/>
+      <c r="E9" s="19" t="n"/>
+      <c r="F9" s="15" t="n"/>
+      <c r="G9" s="15" t="n"/>
+      <c r="H9" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3605,466 +3616,466 @@
   </cols>
   <sheetData>
     <row r="1" ht="29" customHeight="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>산출근거</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
+      <c r="B1" s="15" t="n"/>
+      <c r="C1" s="15" t="n"/>
+      <c r="D1" s="15" t="n"/>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>공사명: 복수 공종 견적</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>기준일: 2026-10-16 | 조건 요약: work_category: 주택 외 건축 (출처: 부문 기본값) · duration: 1~6개월 (출처: 명세 기본값) · contractor_type: 종합건설업 (출처: 명세 기본값) · project_scale: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="n"/>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
+      <c r="A3" s="15" t="inlineStr">
+        <is>
+          <t>기준일: 2026-10-16 | 조건 요약: 공사 종류: 주택 외 건축 (출처: 부문 기본값) · 공사 기간: 1~6개월 (출처: 명세 기본값) · 시공사 업종: 종합건설업 (출처: 명세 기본값) · 전체 공사 규모: 이 견적만 (출처: 명세 기본값) | 부분 산정</t>
+        </is>
+      </c>
+      <c r="B3" s="15" t="n"/>
+      <c r="C3" s="15" t="n"/>
+      <c r="D3" s="15" t="n"/>
     </row>
     <row r="4" ht="27" customHeight="1">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>항목</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>값</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr">
         <is>
           <t>계산</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
         <is>
           <t>근거(품셈 절·표·쪽)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>적용 기준</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr"/>
-      <c r="C5" s="14" t="inlineStr"/>
-      <c r="D5" s="14" t="inlineStr"/>
+      <c r="B5" s="19" t="inlineStr"/>
+      <c r="C5" s="15" t="inlineStr"/>
+      <c r="D5" s="15" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>공사 규모 판정</t>
         </is>
       </c>
-      <c r="B6" s="18" t="inlineStr"/>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr"/>
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>전체 공사 규모: 이 견적만 기준(1,117,900원)으로 제비율 구간을 선택했습니다.</t>
         </is>
       </c>
-      <c r="D6" s="14" t="inlineStr"/>
+      <c r="D6" s="15" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>안전관리비 기초액</t>
         </is>
       </c>
-      <c r="B7" s="18" t="inlineStr"/>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="B7" s="19" t="inlineStr"/>
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>산업안전보건관리비 기초액은 전체 공사에 1회 계상 — 부분 견적에서 제외(간이).</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr"/>
+      <c r="D7" s="15" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 도장공 1㎡당 (인/㎡)</t>
         </is>
       </c>
-      <c r="B8" s="26" t="n">
+      <c r="B8" s="27" t="n">
         <v>0.024</v>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>0.012인 × 1 ÷ 1㎡ × 2회</t>
         </is>
       </c>
-      <c r="D8" s="14" t="inlineStr">
+      <c r="D8" s="15" t="inlineStr">
         <is>
           <t>표 단위당 품 그대로 적용(반올림 없음); 1회 기준 품에 칠 횟수 2회 적용; 11-2-2 p693; 11-2-2 본문 p693</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 보통인부 1㎡당 (인/㎡)</t>
         </is>
       </c>
-      <c r="B9" s="26" t="n">
+      <c r="B9" s="27" t="n">
         <v>0.004</v>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>0.002인 × 1 ÷ 1㎡ × 2회</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>표 단위당 품 그대로 적용(반올림 없음); 1회 기준 품에 칠 횟수 2회 적용; 11-2-2 p693; 11-2-2 본문 p693</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 미산정 범위</t>
         </is>
       </c>
-      <c r="B10" s="18" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>바탕만들기</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>이번 계산 범위에서 미산정</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 미산정 범위</t>
         </is>
       </c>
-      <c r="B11" s="18" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
         <is>
           <t>비계사용시 높이별 품 할증</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="15" t="inlineStr">
         <is>
           <t>이번 계산 범위에서 미산정</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D11" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 미산정 범위</t>
         </is>
       </c>
-      <c r="B12" s="18" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>재료량(페인트 등)</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>이번 계산 범위에서 미산정</t>
         </is>
       </c>
-      <c r="D12" s="14" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 미산정 범위</t>
         </is>
       </c>
-      <c r="B13" s="18" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>바탕만들기</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>PDF 637쪽 11-2-2 [주] ③</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 미산정 범위</t>
         </is>
       </c>
-      <c r="B14" s="18" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>비계사용시 높이별 품 할증</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>PDF 637쪽 11-2-2 [주] ④</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="D14" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 미산정 범위</t>
         </is>
       </c>
-      <c r="B15" s="18" t="inlineStr">
+      <c r="B15" s="19" t="inlineStr">
         <is>
           <t>재료량(페인트 등)</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>PDF 637쪽 11-2-2 [주] ⑥</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 노임 기준 버전</t>
         </is>
       </c>
-      <c r="B16" s="18" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>2026H2</t>
         </is>
       </c>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <t>2026년 하반기 적용 건설업 임금실태조사</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>2026-09-01 ~ 현재</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>[w2_5] 장비 기준 버전</t>
         </is>
       </c>
-      <c r="B17" s="18" t="inlineStr">
+      <c r="B17" s="19" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="C17" s="15" t="inlineStr">
         <is>
           <t>2026년도 건설기계 경비산출표</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D17" s="15" t="inlineStr">
         <is>
           <t>2026-01-01 ~ 2026-12-31</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>[w25_27] 미장공 1㎡당 (인/㎡)</t>
         </is>
       </c>
-      <c r="B18" s="26" t="n">
+      <c r="B18" s="27" t="n">
         <v>0.047</v>
       </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="C18" s="15" t="inlineStr">
         <is>
           <t>0.047인 × 1 ÷ 1㎡</t>
         </is>
       </c>
-      <c r="D18" s="14" t="inlineStr">
+      <c r="D18" s="15" t="inlineStr">
         <is>
           <t>표 단위당 품 그대로 적용(반올림 없음); 6-4-3 p662</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>[w25_27] 보통인부 1㎡당 (인/㎡)</t>
         </is>
       </c>
-      <c r="B19" s="26" t="n">
+      <c r="B19" s="27" t="n">
         <v>0.035</v>
       </c>
-      <c r="C19" s="14" t="inlineStr">
+      <c r="C19" s="15" t="inlineStr">
         <is>
           <t>0.035인 × 1 ÷ 1㎡</t>
         </is>
       </c>
-      <c r="D19" s="14" t="inlineStr">
+      <c r="D19" s="15" t="inlineStr">
         <is>
           <t>표 단위당 품 그대로 적용(반올림 없음); 6-4-3 p662</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>[w25_27] 미산정 범위</t>
         </is>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>모르타르 배합(시멘트, 모래) 재료량</t>
         </is>
       </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>이번 계산 범위에서 미산정</t>
         </is>
       </c>
-      <c r="D20" s="14" t="inlineStr">
+      <c r="D20" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="14" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>[w25_27] 미산정 범위</t>
         </is>
       </c>
-      <c r="B21" s="18" t="inlineStr">
+      <c r="B21" s="19" t="inlineStr">
         <is>
           <t>모르타르 배합(시멘트, 모래) 재료량</t>
         </is>
       </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="C21" s="15" t="inlineStr">
         <is>
           <t>PDF 606쪽 6-4-3 [주] ②</t>
         </is>
       </c>
-      <c r="D21" s="14" t="inlineStr">
+      <c r="D21" s="15" t="inlineStr">
         <is>
           <t>미산정</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>[w25_27] 노임 기준 버전</t>
         </is>
       </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B22" s="19" t="inlineStr">
         <is>
           <t>2026H2</t>
         </is>
       </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="C22" s="15" t="inlineStr">
         <is>
           <t>2026년 하반기 적용 건설업 임금실태조사</t>
         </is>
       </c>
-      <c r="D22" s="14" t="inlineStr">
+      <c r="D22" s="15" t="inlineStr">
         <is>
           <t>2026-09-01 ~ 현재</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="14" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t>[w25_27] 장비 기준 버전</t>
         </is>
       </c>
-      <c r="B23" s="18" t="inlineStr">
+      <c r="B23" s="19" t="inlineStr">
         <is>
           <t>2026</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C23" s="15" t="inlineStr">
         <is>
           <t>2026년도 건설기계 경비산출표</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D23" s="15" t="inlineStr">
         <is>
           <t>2026-01-01 ~ 2026-12-31</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="14" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>통합 제비율 기준 버전</t>
         </is>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B24" s="19" t="inlineStr">
         <is>
           <t>260413</t>
         </is>
       </c>
-      <c r="C24" s="14" t="inlineStr"/>
-      <c r="D24" s="14" t="inlineStr">
+      <c r="C24" s="15" t="inlineStr"/>
+      <c r="D24" s="15" t="inlineStr">
         <is>
           <t>2026-04-13</t>
         </is>
       </c>
     </row>
     <row r="25" ht="23" customHeight="1">
-      <c r="A25" s="25" t="inlineStr">
+      <c r="A25" s="26" t="inlineStr">
         <is>
           <t>표준품셈 기준 금액 · 검토 전 참고용 · 품셈이</t>
         </is>
       </c>
-      <c r="B25" s="18" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
+      <c r="B25" s="19" t="n"/>
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
feat: consolidate calculation coverage, equipment pricing and estimate workflows
</commit_message>
<xml_diff>
--- a/docs/reviews/multi-trade-summary-example.xlsx
+++ b/docs/reviews/multi-trade-summary-example.xlsx
@@ -21,7 +21,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'원가계산서'!$4:$4</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'원가계산서'!$A$1:$E$70</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'내역서'!$4:$5</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'내역서'!$A$1:$M$10</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'내역서'!$A$1:$M$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'일위대가'!$4:$5</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'일위대가'!$A$1:$M$15</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'공종별상세'!$4:$4</definedName>
@@ -2239,7 +2239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2415,7 +2415,7 @@
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>[w2_5] 도장 수성페인트 롤러칠 2회 벽면100㎡ 벽면</t>
+          <t>[w2_5] 도장 수성페인트 롤러칠 2회 벽면100㎡</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
@@ -2461,14 +2461,14 @@
       </c>
       <c r="M6" s="15" t="inlineStr">
         <is>
-          <t>제 1호표 · PARTIAL</t>
+          <t>제 1호표 · PRICED</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>[w25_27] 실내 방수모르타르10㎜ 바닥20㎡ 바닥</t>
+          <t>[w25_27] 실내 방수모르타르10㎜ 바닥20㎡</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="M7" s="15" t="inlineStr">
         <is>
-          <t>제 2호표 · PARTIAL</t>
+          <t>제 2호표 · PRICED</t>
         </is>
       </c>
     </row>
@@ -2555,10 +2555,10 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="29" t="inlineStr">
-        <is>
-          <t>미산정 항목 제외 부분 합계</t>
+    <row r="9" ht="23" customHeight="1">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>표준품셈 기준 금액 · 검토 전 참고용 · 품셈이</t>
         </is>
       </c>
       <c r="B9" s="15" t="n"/>
@@ -2574,27 +2574,8 @@
       <c r="L9" s="19" t="n"/>
       <c r="M9" s="15" t="n"/>
     </row>
-    <row r="10" ht="23" customHeight="1">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>표준품셈 기준 금액 · 검토 전 참고용 · 품셈이</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="n"/>
-      <c r="C10" s="15" t="n"/>
-      <c r="D10" s="19" t="n"/>
-      <c r="E10" s="19" t="n"/>
-      <c r="F10" s="19" t="n"/>
-      <c r="G10" s="19" t="n"/>
-      <c r="H10" s="19" t="n"/>
-      <c r="I10" s="19" t="n"/>
-      <c r="J10" s="19" t="n"/>
-      <c r="K10" s="19" t="n"/>
-      <c r="L10" s="19" t="n"/>
-      <c r="M10" s="15" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="13">
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="I4:J4"/>
@@ -2608,7 +2589,6 @@
     <mergeCell ref="A3:M3"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A10:M10"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.45" bottom="0.45" header="0.2" footer="0.2"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
@@ -2797,7 +2777,7 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>제 1호표 [w2_5] 도장 수성페인트 롤러칠 2회 벽면100㎡ 벽면 (㎡ 당)</t>
+          <t>제 1호표 [w2_5] 도장 수성페인트 롤러칠 2회 벽면100㎡ (㎡ 당)</t>
         </is>
       </c>
       <c r="B6" s="8" t="n"/>
@@ -2931,7 +2911,7 @@
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>제 2호표 [w25_27] 실내 방수모르타르10㎜ 바닥20㎡ 바닥 (㎡ 당)</t>
+          <t>제 2호표 [w25_27] 실내 방수모르타르10㎜ 바닥20㎡ (㎡ 당)</t>
         </is>
       </c>
       <c r="B10" s="15" t="n"/>
@@ -3242,12 +3222,12 @@
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>도장 수성페인트 롤러칠 2회 벽면100㎡ 벽면</t>
+          <t>도장 수성페인트 롤러칠 2회 벽면100㎡</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>PRICED</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
@@ -3283,12 +3263,12 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>실내 방수모르타르10㎜ 바닥20㎡ 바닥</t>
+          <t>실내 방수모르타르10㎜ 바닥20㎡</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>PARTIAL</t>
+          <t>PRICED</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">

</xml_diff>